<commit_message>
docs: record T001 research evaluation
</commit_message>
<xml_diff>
--- a/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
+++ b/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R8c3fe19c4fd046ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="Rb41ae56a44cc48ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="Rd18f44c5dee2439c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R8b4cf47faa8b4038"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="Rc5301e3aceb14a36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="R8c8c3f302c4543ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -277,7 +277,7 @@
         <x:color rgb="FF0F5132"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1E7DD"/>
         </x:patternFill>
       </x:fill>
@@ -288,7 +288,7 @@
         <x:color rgb="FF842029"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF8D7DA"/>
         </x:patternFill>
       </x:fill>
@@ -299,7 +299,7 @@
         <x:color rgb="FF664D03"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3CD"/>
         </x:patternFill>
       </x:fill>
@@ -675,12 +675,12 @@
       <x:c r="B5" s="15"/>
       <x:c r="C5" s="15" t="n">
         <x:f>COUNTIFS('评测记录'!$F$6:$F$10,"已执行")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D5" s="15"/>
       <x:c r="E5" s="16" t="n">
         <x:f>IF(COUNT('评测记录'!$S$6:$S$10)=0,0,AVERAGE('评测记录'!$S$6:$S$10))</x:f>
-        <x:v>0</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="F5" s="16"/>
       <x:c r="G5" s="17" t="n">
@@ -690,12 +690,12 @@
       <x:c r="H5" s="17"/>
       <x:c r="I5" s="15" t="n">
         <x:f>SUM('评测记录'!$P$6:$P$10)</x:f>
-        <x:v>0</x:v>
+        <x:v>42942</x:v>
       </x:c>
       <x:c r="J5" s="15"/>
       <x:c r="K5" s="18" t="n">
         <x:f>SUM('评测记录'!$R$6:$R$10)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.092736</x:v>
       </x:c>
       <x:c r="L5" s="18"/>
       <x:c r="M5" s="1"/>
@@ -1099,18 +1099,18 @@
       <x:c r="V18" s="1"/>
       <x:c r="W18" s="1"/>
     </x:row>
-    <x:row r="19" ht="54" customHeight="1">
+    <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="27" t="str">
-        <x:v>原版基础闭环</x:v>
+        <x:v>原版与首条联网评测</x:v>
       </x:c>
       <x:c r="B19" s="27" t="str">
-        <x:v>启动、登录、DeepSeek 回答、Token 与健康状态</x:v>
+        <x:v>启动、登录、DeepSeek 回答；T001 联网搜索、官方引用和用量记录</x:v>
       </x:c>
       <x:c r="C19" s="27" t="str">
-        <x:v>联网搜索、引用正确性、复杂任务和真实用户价值</x:v>
+        <x:v>完整题集、真实用户价值和生产级可靠性；T001 的时效判断与限制覆盖仍需修正</x:v>
       </x:c>
       <x:c r="D19" s="27" t="str">
-        <x:v>先评测研究质量，不扩张功能</x:v>
+        <x:v>先修正来源时效与限制覆盖，再决定是否扩展到 T002</x:v>
       </x:c>
       <x:c r="E19" s="1"/>
       <x:c r="F19" s="1"/>
@@ -2389,7 +2389,7 @@
         <x:v>复核备注</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="88" customHeight="1">
+    <x:row r="6" ht="150" customHeight="1">
       <x:c r="A6" s="28" t="str">
         <x:v>T001</x:v>
       </x:c>
@@ -2406,38 +2406,65 @@
         <x:v>过期信息、无来源事实、把推断写成事实</x:v>
       </x:c>
       <x:c r="F6" s="44" t="str">
-        <x:v>未执行</x:v>
-      </x:c>
-      <x:c r="G6" s="44"/>
-      <x:c r="H6" s="44"/>
-      <x:c r="I6" s="44"/>
-      <x:c r="J6" s="44"/>
-      <x:c r="K6" s="44"/>
+        <x:v>已执行</x:v>
+      </x:c>
+      <x:c r="G6" s="44" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H6" s="44" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I6" s="44" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J6" s="44" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K6" s="44" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="L6" s="44" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="44" t="str">
-        <x:v>待复核</x:v>
-      </x:c>
-      <x:c r="N6" s="44"/>
-      <x:c r="O6" s="44"/>
-      <x:c r="P6" s="45" t="str">
+        <x:v>需修改</x:v>
+      </x:c>
+      <x:c r="N6" s="44" t="n">
+        <x:v>41800</x:v>
+      </x:c>
+      <x:c r="O6" s="44" t="n">
+        <x:v>1142</x:v>
+      </x:c>
+      <x:c r="P6" s="45" t="n">
         <x:f>IF(COUNT(N6:O6)=0,"",SUM(N6:O6))</x:f>
-      </x:c>
-      <x:c r="Q6" s="44"/>
-      <x:c r="R6" s="46" t="str">
+        <x:v>42942</x:v>
+      </x:c>
+      <x:c r="Q6" s="44" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="R6" s="46" t="n">
         <x:f>IF(F6&lt;&gt;"已执行","",N6*'概览'!$B$9/1000000+O6*'概览'!$C$9/1000000)</x:f>
-      </x:c>
-      <x:c r="S6" s="47" t="str">
+        <x:v>0.092736</x:v>
+      </x:c>
+      <x:c r="S6" s="47" t="n">
         <x:f>IF(COUNT(G6:K6)&lt;5,"",(G6*'评分标准'!$B$4+H6*'评分标准'!$B$5+I6*'评分标准'!$B$6+J6*'评分标准'!$B$7+K6*'评分标准'!$B$8)/5*100)</x:f>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="T6" s="45" t="str">
         <x:f>IF(F6&lt;&gt;"已执行","待执行",IF(L6&gt;0,"失败",IF(M6="失败","失败",IF(M6="需修改","需改进",IF(M6&lt;&gt;"通过","待人工复核",IF(S6&gt;=80,"通过","需改进"))))))</x:f>
-        <x:v>待执行</x:v>
-      </x:c>
-      <x:c r="U6" s="40" t="str"/>
-      <x:c r="V6" s="40" t="str"/>
-      <x:c r="W6" s="40" t="str"/>
+        <x:v>需改进</x:v>
+      </x:c>
+      <x:c r="U6" s="40" t="str">
+        <x:v>引用均来自官方页面，但把发布时的 o3 与 o4-mini 机制写成当前事实；遗漏同页已披露的幻觉、错误推断、权威来源识别和置信度校准限制；“未找到量化指标”与同页 26.6% 基准信息冲突。</x:v>
+      </x:c>
+      <x:c r="V6" s="40" t="str">
+        <x:v>http://localhost:2026/workspace/chats/bed321a8-d6eb-4a57-9a70-6bbb5f59f3f3
+https://openai.com/index/introducing-deep-research/
+https://help.openai.com/en/articles/10500283-deep-research-in-chatgpt</x:v>
+      </x:c>
+      <x:c r="W6" s="40" t="str">
+        <x:v>Codex 辅助人工复核，2026-09-19。2 次搜索、3 次查看、2 个唯一官方页面；未见第三方来源或子智能体。主回复输入约 41.8K、输出 1,142；线程顶部总量 43.2K。延迟约 17 秒。正文含 494 个汉字，总字符约 1,287。</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="88" customHeight="1">
       <x:c r="A7" s="28" t="str">
@@ -3935,7 +3962,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12e3a4ae6327417a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3eeb32ea19f4295"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs: strengthen research quality gates
</commit_message>
<xml_diff>
--- a/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
+++ b/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R8b4cf47faa8b4038"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="Rc5301e3aceb14a36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="R8c8c3f302c4543ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R177ff51167194185"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="R89aa87e536d64291"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="Rb54f071bdc1f4239"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +22,7 @@
     <x:numFmt numFmtId="203" formatCode="0.000000"/>
     <x:numFmt numFmtId="204" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -67,8 +67,14 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -108,6 +114,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF275D85"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -159,7 +175,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -265,6 +281,20 @@
     </x:xf>
     <x:xf numFmtId="204" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1101,16 +1131,16 @@
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="27" t="str">
-        <x:v>原版与首条联网评测</x:v>
+        <x:v>原版、T001 与质量门禁</x:v>
       </x:c>
       <x:c r="B19" s="27" t="str">
-        <x:v>启动、登录、DeepSeek 回答；T001 联网搜索、官方引用和用量记录</x:v>
+        <x:v>原版闭环、T001 联网评测；研究质量门禁 v1.1 已固化</x:v>
       </x:c>
       <x:c r="C19" s="27" t="str">
-        <x:v>完整题集、真实用户价值和生产级可靠性；T001 的时效判断与限制覆盖仍需修正</x:v>
+        <x:v>T001 v2 重测、完整题集、真实用户价值和生产级可靠性</x:v>
       </x:c>
       <x:c r="D19" s="27" t="str">
-        <x:v>先修正来源时效与限制覆盖，再决定是否扩展到 T002</x:v>
+        <x:v>先用现有 Badcase 走查门禁；获新费用授权后再决定是否重跑</x:v>
       </x:c>
       <x:c r="E19" s="1"/>
       <x:c r="F19" s="1"/>
@@ -3962,7 +3992,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3eeb32ea19f4295"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5300a3b71fe54d27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3975,7 +4005,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
@@ -4011,7 +4041,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>总分 100；0—5 分由人工依据证据评分。任何高风险无依据结论都会直接导致发布闸门失败。</x:v>
+        <x:v>总分 100；0—5 分由人工依据证据评分。当前状态仅由历史资料支持、关键引用不支持结论或高风险无依据结论，均不得通过。</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -4081,16 +4111,16 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="C4" s="27" t="str">
-        <x:v>关键事实与来源一致，来源可访问且时效明确</x:v>
+        <x:v>当前事实由当前官方文档支持；历史资料标注时间；来源可访问</x:v>
       </x:c>
       <x:c r="D4" s="27" t="str">
-        <x:v>少量一般事实需修正，不影响主要结论</x:v>
+        <x:v>少量一般事实时效或表述需修正，不影响主要结论</x:v>
       </x:c>
       <x:c r="E4" s="27" t="str">
-        <x:v>关键事实错误、来源失效或来源与结论不符</x:v>
+        <x:v>关键事实错误、历史信息冒充当前状态或来源与结论不符</x:v>
       </x:c>
       <x:c r="F4" s="27" t="str">
-        <x:v>逐条抽查关键事实</x:v>
+        <x:v>先查当前文档，再核历史页面的时间语境</x:v>
       </x:c>
       <x:c r="G4" s="1"/>
       <x:c r="H4" s="1"/>
@@ -4118,16 +4148,16 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="C5" s="27" t="str">
-        <x:v>所有关键结论有来源，一般事实覆盖率不低于90%</x:v>
+        <x:v>关键结论 100% 有直接支持链接，一般事实覆盖率不低于 90%</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>主要结论有来源，仍有明显缺口</x:v>
+        <x:v>主要结论有来源，但仍有定位或支持关系缺口</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
-        <x:v>大量结论无来源或引用无法定位</x:v>
+        <x:v>大量结论无来源，或链接存在但不支持对应结论</x:v>
       </x:c>
       <x:c r="F5" s="27" t="str">
-        <x:v>关键结论必须100%覆盖</x:v>
+        <x:v>逐条验证结论与引用内容的一致性</x:v>
       </x:c>
       <x:c r="G5" s="1"/>
       <x:c r="H5" s="1"/>
@@ -4155,16 +4185,16 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="C6" s="27" t="str">
-        <x:v>按要求覆盖全部维度，并标注冲突与未知</x:v>
+        <x:v>覆盖能力、范围、限制/失败模式、使用规则和日期，并标注冲突与未知</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
-        <x:v>覆盖主要维度，但遗漏部分限制或冲突</x:v>
+        <x:v>覆盖主要维度，但遗漏部分限制、量化信息或冲突</x:v>
       </x:c>
       <x:c r="E6" s="27" t="str">
-        <x:v>结构缺失，无法支持产品判断</x:v>
+        <x:v>只写能力优点，结构缺失，无法支持产品判断</x:v>
       </x:c>
       <x:c r="F6" s="27" t="str">
-        <x:v>检查未知项是否被强行补齐</x:v>
+        <x:v>主动检查 limitations、usage、availability、updated</x:v>
       </x:c>
       <x:c r="G6" s="1"/>
       <x:c r="H6" s="1"/>
@@ -4192,16 +4222,16 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="C7" s="27" t="str">
-        <x:v>范围、格式、字数和来源要求全部满足</x:v>
+        <x:v>来源、搜索/页面上限、工具、总字符数和输出结构全部满足</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
-        <x:v>存在轻微偏离，但输出仍可使用</x:v>
+        <x:v>存在轻微偏离，但输出仍可复核使用</x:v>
       </x:c>
       <x:c r="E7" s="27" t="str">
-        <x:v>违反关键限制或自行扩大任务</x:v>
+        <x:v>使用禁止来源、越界工具、超出关键范围或自行扩张任务</x:v>
       </x:c>
       <x:c r="F7" s="27" t="str">
-        <x:v>检查是否使用禁止来源或越界事实</x:v>
+        <x:v>长度按总字符计算，不只统计汉字</x:v>
       </x:c>
       <x:c r="G7" s="1"/>
       <x:c r="H7" s="1"/>
@@ -4229,16 +4259,16 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="C8" s="27" t="str">
-        <x:v>结论清晰、可复核，可直接支持下一步人工决策</x:v>
+        <x:v>事实、历史信息、推断、建议和未知清晰分开，可直接支持人工决策</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
-        <x:v>需要编辑后才能用于评审</x:v>
+        <x:v>需要明显编辑后才能用于评审</x:v>
       </x:c>
       <x:c r="E8" s="27" t="str">
-        <x:v>信息堆砌，无法形成行动判断</x:v>
+        <x:v>信息堆砌或混淆事实与判断，无法形成行动结论</x:v>
       </x:c>
       <x:c r="F8" s="27" t="str">
-        <x:v>产品建议必须区分事实与推断</x:v>
+        <x:v>复核结论必须明确为通过、需修改或失败</x:v>
       </x:c>
       <x:c r="G8" s="1"/>
       <x:c r="H8" s="1"/>
@@ -4804,13 +4834,15 @@
       <x:c r="V26" s="1"/>
       <x:c r="W26" s="1"/>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="1"/>
-      <x:c r="B27" s="1"/>
-      <x:c r="C27" s="1"/>
-      <x:c r="D27" s="1"/>
-      <x:c r="E27" s="1"/>
-      <x:c r="F27" s="1"/>
+    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="A27" s="52" t="str">
+        <x:v>研究质量门禁 v1.1</x:v>
+      </x:c>
+      <x:c r="B27" s="52"/>
+      <x:c r="C27" s="52"/>
+      <x:c r="D27" s="52"/>
+      <x:c r="E27" s="52"/>
+      <x:c r="F27" s="52"/>
       <x:c r="G27" s="1"/>
       <x:c r="H27" s="1"/>
       <x:c r="I27" s="1"/>
@@ -4830,12 +4862,24 @@
       <x:c r="W27" s="1"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="1"/>
-      <x:c r="B28" s="1"/>
-      <x:c r="C28" s="1"/>
-      <x:c r="D28" s="1"/>
-      <x:c r="E28" s="1"/>
-      <x:c r="F28" s="1"/>
+      <x:c r="A28" s="57" t="str">
+        <x:v>编号</x:v>
+      </x:c>
+      <x:c r="B28" s="57" t="str">
+        <x:v>门禁</x:v>
+      </x:c>
+      <x:c r="C28" s="57" t="str">
+        <x:v>通过条件</x:v>
+      </x:c>
+      <x:c r="D28" s="57" t="str">
+        <x:v>失败示例</x:v>
+      </x:c>
+      <x:c r="E28" s="57" t="str">
+        <x:v>处理</x:v>
+      </x:c>
+      <x:c r="F28" s="57" t="str">
+        <x:v>人工复核重点</x:v>
+      </x:c>
       <x:c r="G28" s="1"/>
       <x:c r="H28" s="1"/>
       <x:c r="I28" s="1"/>
@@ -4854,13 +4898,25 @@
       <x:c r="V28" s="1"/>
       <x:c r="W28" s="1"/>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="1"/>
-      <x:c r="B29" s="1"/>
-      <x:c r="C29" s="1"/>
-      <x:c r="D29" s="1"/>
-      <x:c r="E29" s="1"/>
-      <x:c r="F29" s="1"/>
+    <x:row r="29" ht="62" customHeight="1">
+      <x:c r="A29" s="28" t="str">
+        <x:v>QG-01</x:v>
+      </x:c>
+      <x:c r="B29" s="27" t="str">
+        <x:v>当前性</x:v>
+      </x:c>
+      <x:c r="C29" s="27" t="str">
+        <x:v>当前状态优先当前官方文档；历史信息标注日期或“发布时”</x:v>
+      </x:c>
+      <x:c r="D29" s="27" t="str">
+        <x:v>把发布时模型写成当前模型</x:v>
+      </x:c>
+      <x:c r="E29" s="27" t="str">
+        <x:v>需修改</x:v>
+      </x:c>
+      <x:c r="F29" s="27" t="str">
+        <x:v>核对页面类型、发布日期和访问日期</x:v>
+      </x:c>
       <x:c r="G29" s="1"/>
       <x:c r="H29" s="1"/>
       <x:c r="I29" s="1"/>
@@ -4879,13 +4935,25 @@
       <x:c r="V29" s="1"/>
       <x:c r="W29" s="1"/>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="1"/>
-      <x:c r="B30" s="1"/>
-      <x:c r="C30" s="1"/>
-      <x:c r="D30" s="1"/>
-      <x:c r="E30" s="1"/>
-      <x:c r="F30" s="1"/>
+    <x:row r="30" ht="62" customHeight="1">
+      <x:c r="A30" s="28" t="str">
+        <x:v>QG-02</x:v>
+      </x:c>
+      <x:c r="B30" s="27" t="str">
+        <x:v>证据一致性</x:v>
+      </x:c>
+      <x:c r="C30" s="27" t="str">
+        <x:v>每条关键结论都有直接支持它的证据</x:v>
+      </x:c>
+      <x:c r="D30" s="27" t="str">
+        <x:v>链接存在但页面不支持结论</x:v>
+      </x:c>
+      <x:c r="E30" s="27" t="str">
+        <x:v>需修改或失败</x:v>
+      </x:c>
+      <x:c r="F30" s="27" t="str">
+        <x:v>逐条对照结论与原文含义</x:v>
+      </x:c>
       <x:c r="G30" s="1"/>
       <x:c r="H30" s="1"/>
       <x:c r="I30" s="1"/>
@@ -4904,13 +4972,25 @@
       <x:c r="V30" s="1"/>
       <x:c r="W30" s="1"/>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="1"/>
-      <x:c r="B31" s="1"/>
-      <x:c r="C31" s="1"/>
-      <x:c r="D31" s="1"/>
-      <x:c r="E31" s="1"/>
-      <x:c r="F31" s="1"/>
+    <x:row r="31" ht="62" customHeight="1">
+      <x:c r="A31" s="28" t="str">
+        <x:v>QG-03</x:v>
+      </x:c>
+      <x:c r="B31" s="27" t="str">
+        <x:v>引用覆盖</x:v>
+      </x:c>
+      <x:c r="C31" s="27" t="str">
+        <x:v>关键结论覆盖率 100%，一般事实不低于 90%</x:v>
+      </x:c>
+      <x:c r="D31" s="27" t="str">
+        <x:v>核心能力或限制没有来源</x:v>
+      </x:c>
+      <x:c r="E31" s="27" t="str">
+        <x:v>需修改</x:v>
+      </x:c>
+      <x:c r="F31" s="27" t="str">
+        <x:v>先检查关键结论</x:v>
+      </x:c>
       <x:c r="G31" s="1"/>
       <x:c r="H31" s="1"/>
       <x:c r="I31" s="1"/>
@@ -4929,13 +5009,25 @@
       <x:c r="V31" s="1"/>
       <x:c r="W31" s="1"/>
     </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="1"/>
-      <x:c r="B32" s="1"/>
-      <x:c r="C32" s="1"/>
-      <x:c r="D32" s="1"/>
-      <x:c r="E32" s="1"/>
-      <x:c r="F32" s="1"/>
+    <x:row r="32" ht="62" customHeight="1">
+      <x:c r="A32" s="28" t="str">
+        <x:v>QG-04</x:v>
+      </x:c>
+      <x:c r="B32" s="27" t="str">
+        <x:v>限制完整性</x:v>
+      </x:c>
+      <x:c r="C32" s="27" t="str">
+        <x:v>覆盖限制、失败模式、额度、可用性和量化评测</x:v>
+      </x:c>
+      <x:c r="D32" s="27" t="str">
+        <x:v>只写优点，遗漏幻觉或错误推断</x:v>
+      </x:c>
+      <x:c r="E32" s="27" t="str">
+        <x:v>需修改</x:v>
+      </x:c>
+      <x:c r="F32" s="27" t="str">
+        <x:v>主动寻找不利信息</x:v>
+      </x:c>
       <x:c r="G32" s="1"/>
       <x:c r="H32" s="1"/>
       <x:c r="I32" s="1"/>
@@ -4954,13 +5046,25 @@
       <x:c r="V32" s="1"/>
       <x:c r="W32" s="1"/>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="1"/>
-      <x:c r="B33" s="1"/>
-      <x:c r="C33" s="1"/>
-      <x:c r="D33" s="1"/>
-      <x:c r="E33" s="1"/>
-      <x:c r="F33" s="1"/>
+    <x:row r="33" ht="62" customHeight="1">
+      <x:c r="A33" s="28" t="str">
+        <x:v>QG-05</x:v>
+      </x:c>
+      <x:c r="B33" s="27" t="str">
+        <x:v>冲突与未知</x:v>
+      </x:c>
+      <x:c r="C33" s="27" t="str">
+        <x:v>冲突并列；无法确认写未知，不自行补全</x:v>
+      </x:c>
+      <x:c r="D33" s="27" t="str">
+        <x:v>擅自裁决冲突或把未找到写成不存在</x:v>
+      </x:c>
+      <x:c r="E33" s="27" t="str">
+        <x:v>需修改</x:v>
+      </x:c>
+      <x:c r="F33" s="27" t="str">
+        <x:v>检查否定性结论的证据</x:v>
+      </x:c>
       <x:c r="G33" s="1"/>
       <x:c r="H33" s="1"/>
       <x:c r="I33" s="1"/>
@@ -4979,13 +5083,25 @@
       <x:c r="V33" s="1"/>
       <x:c r="W33" s="1"/>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="1"/>
-      <x:c r="B34" s="1"/>
-      <x:c r="C34" s="1"/>
-      <x:c r="D34" s="1"/>
-      <x:c r="E34" s="1"/>
-      <x:c r="F34" s="1"/>
+    <x:row r="34" ht="62" customHeight="1">
+      <x:c r="A34" s="28" t="str">
+        <x:v>QG-06</x:v>
+      </x:c>
+      <x:c r="B34" s="27" t="str">
+        <x:v>范围与成本</x:v>
+      </x:c>
+      <x:c r="C34" s="27" t="str">
+        <x:v>满足搜索、页面、工具、时间和总字符数限制</x:v>
+      </x:c>
+      <x:c r="D34" s="27" t="str">
+        <x:v>无限搜索、启用子智能体或超长输出</x:v>
+      </x:c>
+      <x:c r="E34" s="27" t="str">
+        <x:v>停止并复盘</x:v>
+      </x:c>
+      <x:c r="F34" s="27" t="str">
+        <x:v>记录实际 Token、延迟和费用</x:v>
+      </x:c>
       <x:c r="G34" s="1"/>
       <x:c r="H34" s="1"/>
       <x:c r="I34" s="1"/>
@@ -5004,13 +5120,25 @@
       <x:c r="V34" s="1"/>
       <x:c r="W34" s="1"/>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="1"/>
-      <x:c r="B35" s="1"/>
-      <x:c r="C35" s="1"/>
-      <x:c r="D35" s="1"/>
-      <x:c r="E35" s="1"/>
-      <x:c r="F35" s="1"/>
+    <x:row r="35" ht="62" customHeight="1">
+      <x:c r="A35" s="28" t="str">
+        <x:v>QG-07</x:v>
+      </x:c>
+      <x:c r="B35" s="27" t="str">
+        <x:v>可审计性</x:v>
+      </x:c>
+      <x:c r="C35" s="27" t="str">
+        <x:v>保存访问日期、模型、Token、费用、证据路径和人工结论</x:v>
+      </x:c>
+      <x:c r="D35" s="27" t="str">
+        <x:v>只有答案，无法复盘</x:v>
+      </x:c>
+      <x:c r="E35" s="27" t="str">
+        <x:v>不得进入下一阶段</x:v>
+      </x:c>
+      <x:c r="F35" s="27" t="str">
+        <x:v>证据记录完整且可打开</x:v>
+      </x:c>
       <x:c r="G35" s="1"/>
       <x:c r="H35" s="1"/>
       <x:c r="I35" s="1"/>
@@ -5658,6 +5786,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A27:F27"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record T001 v2 regression
</commit_message>
<xml_diff>
--- a/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
+++ b/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R177ff51167194185"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="R89aa87e536d64291"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="Rb54f071bdc1f4239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Rf53485809d7c40bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="Rbf21f715c4744f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="R2ef8146c7792491c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,7 +74,7 @@
       <x:name val="Microsoft YaHei"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -126,6 +126,16 @@
         <x:fgColor rgb="FF275D85"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="4">
     <x:border/>
@@ -175,7 +185,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="66">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -296,11 +306,35 @@
     <x:xf numFmtId="0" fontId="6" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="6">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -334,12 +368,45 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF0F5132"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD1E7DD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF842029"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF8D7DA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF664D03"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF3CD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvaluationTasks" displayName="EvaluationTasks" ref="A5:W10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvaluationTasks" displayName="EvaluationTasks" ref="A5:W11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="23">
     <x:tableColumn id="1" name="任务ID"/>
     <x:tableColumn id="2" name="用户场景"/>
@@ -610,7 +677,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>本表中的 5 条任务均为合成评测题，不代表真实用户、真实客户或生产数据。</x:v>
+        <x:v>本表记录 5 个合成题型及其回归运行，不代表真实用户、真实客户或生产数据。</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -662,7 +729,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="str">
-        <x:v>任务总数</x:v>
+        <x:v>评测记录数</x:v>
       </x:c>
       <x:c r="B4" s="10" t="str"/>
       <x:c r="C4" s="10" t="str">
@@ -699,33 +766,33 @@
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="15" t="n">
-        <x:f>COUNTA('评测记录'!$A$6:$A$10)</x:f>
-        <x:v>5</x:v>
+        <x:f>COUNTA('评测记录'!$A$6:$A$11)</x:f>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B5" s="15"/>
       <x:c r="C5" s="15" t="n">
-        <x:f>COUNTIFS('评测记录'!$F$6:$F$10,"已执行")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIFS('评测记录'!$F$6:$F$11,"已执行")</x:f>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="15"/>
       <x:c r="E5" s="16" t="n">
-        <x:f>IF(COUNT('评测记录'!$S$6:$S$10)=0,0,AVERAGE('评测记录'!$S$6:$S$10))</x:f>
-        <x:v>67</x:v>
+        <x:f>IF(COUNT('评测记录'!$S$6:$S$11)=0,0,AVERAGE('评测记录'!$S$6:$S$11))</x:f>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="F5" s="16"/>
       <x:c r="G5" s="17" t="n">
-        <x:f>IF(COUNTIFS('评测记录'!$F$6:$F$10,"已执行")=0,0,COUNTIFS('评测记录'!$T$6:$T$10,"通过")/COUNTIFS('评测记录'!$F$6:$F$10,"已执行"))</x:f>
+        <x:f>IF(COUNTIFS('评测记录'!$F$6:$F$11,"已执行")=0,0,COUNTIFS('评测记录'!$T$6:$T$11,"通过")/COUNTIFS('评测记录'!$F$6:$F$11,"已执行"))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="17"/>
       <x:c r="I5" s="15" t="n">
-        <x:f>SUM('评测记录'!$P$6:$P$10)</x:f>
-        <x:v>42942</x:v>
+        <x:f>SUM('评测记录'!$P$6:$P$11)</x:f>
+        <x:v>76242</x:v>
       </x:c>
       <x:c r="J5" s="15"/>
       <x:c r="K5" s="18" t="n">
-        <x:f>SUM('评测记录'!$R$6:$R$10)</x:f>
-        <x:v>0.092736</x:v>
+        <x:f>SUM('评测记录'!$R$6:$R$11)</x:f>
+        <x:v>0.164736</x:v>
       </x:c>
       <x:c r="L5" s="18"/>
       <x:c r="M5" s="1"/>
@@ -1131,16 +1198,16 @@
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="27" t="str">
-        <x:v>原版、T001 与质量门禁</x:v>
+        <x:v>T001 v2 回归完成</x:v>
       </x:c>
       <x:c r="B19" s="27" t="str">
-        <x:v>原版闭环、T001 联网评测；研究质量门禁 v1.1 已固化</x:v>
+        <x:v>质量门禁改善了时效标注、结构、成本和长度；得分由 67 升至 79</x:v>
       </x:c>
       <x:c r="C19" s="27" t="str">
-        <x:v>T001 v2 重测、完整题集、真实用户价值和生产级可靠性</x:v>
+        <x:v>仍遗漏模型质量限制，并出现无依据的 Pro $200 暂停注册前提</x:v>
       </x:c>
       <x:c r="D19" s="27" t="str">
-        <x:v>先用现有 Badcase 走查门禁；获新费用授权后再决定是否重跑</x:v>
+        <x:v>保持需改进，不扩展 T002；先修正未知项与限制提取规则</x:v>
       </x:c>
       <x:c r="E19" s="1"/>
       <x:c r="F19" s="1"/>
@@ -2263,7 +2330,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>黄色列为人工填写；蓝色列为自动计算。5 条任务为合成案例，不是生产数据。</x:v>
+        <x:v>黄色列为人工填写；蓝色列为自动计算。当前包含 5 个合成题型和回归运行，不是生产数据。</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2696,30 +2763,83 @@
       <x:c r="V10" s="40" t="str"/>
       <x:c r="W10" s="40" t="str"/>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="1"/>
-      <x:c r="B11" s="1"/>
-      <x:c r="C11" s="1"/>
-      <x:c r="D11" s="1"/>
-      <x:c r="E11" s="1"/>
-      <x:c r="F11" s="1"/>
-      <x:c r="G11" s="1"/>
-      <x:c r="H11" s="1"/>
-      <x:c r="I11" s="1"/>
-      <x:c r="J11" s="1"/>
-      <x:c r="K11" s="1"/>
-      <x:c r="L11" s="1"/>
-      <x:c r="M11" s="1"/>
-      <x:c r="N11" s="1"/>
-      <x:c r="O11" s="1"/>
-      <x:c r="P11" s="1"/>
-      <x:c r="Q11" s="1"/>
-      <x:c r="R11" s="1"/>
-      <x:c r="S11" s="1"/>
-      <x:c r="T11" s="1"/>
-      <x:c r="U11" s="1"/>
-      <x:c r="V11" s="1"/>
-      <x:c r="W11" s="1"/>
+    <x:row r="11" ht="150" customHeight="1">
+      <x:c r="A11" s="28" t="str">
+        <x:v>T001-v2</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="str">
+        <x:v>质量门禁修正后的回归评测</x:v>
+      </x:c>
+      <x:c r="C11" s="27" t="str">
+        <x:v>按 RESEARCH_QUALITY_GATES.md 的 T001 v2 指令，限制为 2 次搜索、3 个唯一官方页面和 800 个总字符；当前文档优先，历史信息标时，覆盖限制与未知。</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="str">
+        <x:v>当前事实、历史信息、主要限制、待人工复核项</x:v>
+      </x:c>
+      <x:c r="E11" s="27" t="str">
+        <x:v>历史信息冒充当前、限制遗漏、无依据未知项</x:v>
+      </x:c>
+      <x:c r="F11" s="62" t="str">
+        <x:v>已执行</x:v>
+      </x:c>
+      <x:c r="G11" s="62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H11" s="62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I11" s="62" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J11" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K11" s="62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L11" s="62" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M11" s="62" t="str">
+        <x:v>需修改</x:v>
+      </x:c>
+      <x:c r="N11" s="62" t="n">
+        <x:v>32400</x:v>
+      </x:c>
+      <x:c r="O11" s="62" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="P11" s="63" t="n">
+        <x:f>IF(COUNT(N11:O11)=0,"",SUM(N11:O11))</x:f>
+        <x:v>33300</x:v>
+      </x:c>
+      <x:c r="Q11" s="62" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="R11" s="64" t="n">
+        <x:f>IF(F11&lt;&gt;"已执行","",N11*'概览'!$B$9/1000000+O11*'概览'!$C$9/1000000)</x:f>
+        <x:v>0.072</x:v>
+      </x:c>
+      <x:c r="S11" s="65" t="n">
+        <x:f>IF(COUNT(G11:K11)&lt;5,"",(G11*'评分标准'!$B$4+H11*'评分标准'!$B$5+I11*'评分标准'!$B$6+J11*'评分标准'!$B$7+K11*'评分标准'!$B$8)/5*100)</x:f>
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="T11" s="63" t="str">
+        <x:f>IF(F11&lt;&gt;"已执行","待执行",IF(L11&gt;0,"失败",IF(M11="失败","失败",IF(M11="需修改","需改进",IF(M11&lt;&gt;"通过","待人工复核",IF(S11&gt;=80,"通过","需改进"))))))</x:f>
+        <x:v>需改进</x:v>
+      </x:c>
+      <x:c r="U11" s="58" t="str">
+        <x:v>历史信息已正确分区，当前用量、可用性和权限限制有直接引用；但仍遗漏发布页明确的幻觉、错误推断、权威来源识别和置信度校准问题；“Pro $200 暂停注册”无所读官方页面支持。</x:v>
+      </x:c>
+      <x:c r="V11" s="58" t="str">
+        <x:v>http://localhost:2026/workspace/chats/a58c5f86-f156-476d-af45-24c12a78c8c5
+https://help.openai.com/en/articles/10500283-deep-research-in-chatgpt
+https://help.openai.com/en/articles/6825453-chatgpt-release-notes
+https://openai.com/index/introducing-deep-research/</x:v>
+      </x:c>
+      <x:c r="W11" s="58" t="str">
+        <x:v>Codex 辅助人工复核，2026-09-19。2 次搜索、3 次查看、3 个唯一官方页面；未见第三方来源、子智能体或文件生成。主回复输入约 32.4K、输出 900；线程顶部输入 32.7K、输出 909、总量 33.6K。延迟约 10 秒，正文 575 个总字符。较 v1 得分增加 12，主回复成本约下降 22%，正文长度约下降 55%。</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1"/>
@@ -3968,7 +4088,24 @@
     <x:cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="失败"/>
     <x:cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="需改进"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="6">
+  <x:conditionalFormatting sqref="S11:S11">
+    <x:cfRule type="colorScale" priority="5">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8D7DA"/>
+        <x:color rgb="FFFFF3CD"/>
+        <x:color rgb="FFD1E7DD"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="T11:T11">
+    <x:cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="通过"/>
+    <x:cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="失败"/>
+    <x:cfRule type="containsText" dxfId="5" priority="8" operator="containsText" text="需改进"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="12">
     <x:dataValidation type="list" sqref="F6:F10">
       <x:formula1>"未执行,已执行"</x:formula1>
     </x:dataValidation>
@@ -3989,10 +4126,30 @@
     <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="Q6:Q10">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="F11">
+      <x:formula1>"未执行,已执行"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="G11:K11">
+      <x:formula1>0</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="L11">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="M11">
+      <x:formula1>"待复核,通过,需修改,失败"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="N11:O11">
+      <x:formula1>0</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="Q11">
+      <x:formula1>0</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5300a3b71fe54d27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc2dc99f63004fc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs: refine research quality gates v1.2
</commit_message>
<xml_diff>
--- a/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
+++ b/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Rf53485809d7c40bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="Rbf21f715c4744f1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="R2ef8146c7792491c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R366e3e5910494b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="R7b4314fb6ef04914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="R11cd880bd93e498a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -374,7 +374,7 @@
         <x:color rgb="FF0F5132"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1E7DD"/>
         </x:patternFill>
       </x:fill>
@@ -385,7 +385,7 @@
         <x:color rgb="FF842029"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF8D7DA"/>
         </x:patternFill>
       </x:fill>
@@ -396,7 +396,7 @@
         <x:color rgb="FF664D03"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3CD"/>
         </x:patternFill>
       </x:fill>
@@ -1198,16 +1198,16 @@
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="27" t="str">
-        <x:v>T001 v2 回归完成</x:v>
+        <x:v>质量门禁 v1.2 已修正</x:v>
       </x:c>
       <x:c r="B19" s="27" t="str">
-        <x:v>质量门禁改善了时效标注、结构、成本和长度；得分由 67 升至 79</x:v>
+        <x:v>补充未知项前提检查，并强制区分操作限制与模型质量限制</x:v>
       </x:c>
       <x:c r="C19" s="27" t="str">
-        <x:v>仍遗漏模型质量限制，并出现无依据的 Pro $200 暂停注册前提</x:v>
+        <x:v>T001 v3 尚未运行，v1.2 仅完成规则级验证</x:v>
       </x:c>
       <x:c r="D19" s="27" t="str">
-        <x:v>保持需改进，不扩展 T002；先修正未知项与限制提取规则</x:v>
+        <x:v>不执行 T002；获得新费用授权后再决定是否运行 T001 v3</x:v>
       </x:c>
       <x:c r="E19" s="1"/>
       <x:c r="F19" s="1"/>
@@ -4149,7 +4149,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc2dc99f63004fc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc0185037b7e4497"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4198,7 +4198,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>总分 100；0—5 分由人工依据证据评分。当前状态仅由历史资料支持、关键引用不支持结论或高风险无依据结论，均不得通过。</x:v>
+        <x:v>总分 100；0—5 分由人工依据证据评分。当前状态仅由历史资料支持、任何陈述含无依据前提、关键引用不支持结论或高风险无依据结论，均不得通过。</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -4305,16 +4305,16 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="C5" s="27" t="str">
-        <x:v>关键结论 100% 有直接支持链接，一般事实覆盖率不低于 90%</x:v>
+        <x:v>关键结论及待复核项中的事实前提 100% 有直接支持链接，一般事实覆盖率不低于 90%</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>主要结论有来源，但仍有定位或支持关系缺口</x:v>
+        <x:v>主要结论有来源，但仍有定位、支持关系或待复核项证据缺口</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
         <x:v>大量结论无来源，或链接存在但不支持对应结论</x:v>
       </x:c>
       <x:c r="F5" s="27" t="str">
-        <x:v>逐条验证结论与引用内容的一致性</x:v>
+        <x:v>逐条验证结论和待复核项前提与引用内容的一致性</x:v>
       </x:c>
       <x:c r="G5" s="1"/>
       <x:c r="H5" s="1"/>
@@ -4342,16 +4342,16 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="C6" s="27" t="str">
-        <x:v>覆盖能力、范围、限制/失败模式、使用规则和日期，并标注冲突与未知</x:v>
+        <x:v>覆盖能力、范围、操作限制、模型质量失败模式、使用规则和日期，并标注冲突与未知</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
-        <x:v>覆盖主要维度，但遗漏部分限制、量化信息或冲突</x:v>
+        <x:v>覆盖主要维度，但遗漏部分模型质量限制、量化信息或冲突</x:v>
       </x:c>
       <x:c r="E6" s="27" t="str">
-        <x:v>只写能力优点，结构缺失，无法支持产品判断</x:v>
+        <x:v>只写能力与操作限制，遗漏官方已披露的模型质量失败模式</x:v>
       </x:c>
       <x:c r="F6" s="27" t="str">
-        <x:v>主动检查 limitations、usage、availability、updated</x:v>
+        <x:v>若官方已披露，至少提取 2 项模型质量失败模式</x:v>
       </x:c>
       <x:c r="G6" s="1"/>
       <x:c r="H6" s="1"/>
@@ -4416,16 +4416,16 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="C8" s="27" t="str">
-        <x:v>事实、历史信息、推断、建议和未知清晰分开，可直接支持人工决策</x:v>
+        <x:v>事实、历史信息、推断、建议和未知清晰分开；待复核项不引入新事实前提</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
         <x:v>需要明显编辑后才能用于评审</x:v>
       </x:c>
       <x:c r="E8" s="27" t="str">
-        <x:v>信息堆砌或混淆事实与判断，无法形成行动结论</x:v>
+        <x:v>混淆事实与判断，或用无依据前提制造待复核项</x:v>
       </x:c>
       <x:c r="F8" s="27" t="str">
-        <x:v>复核结论必须明确为通过、需修改或失败</x:v>
+        <x:v>检查未知项是否为中性问题，而非暗含未经证实事件</x:v>
       </x:c>
       <x:c r="G8" s="1"/>
       <x:c r="H8" s="1"/>
@@ -4993,7 +4993,7 @@
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
       <x:c r="A27" s="52" t="str">
-        <x:v>研究质量门禁 v1.1</x:v>
+        <x:v>研究质量门禁 v1.2</x:v>
       </x:c>
       <x:c r="B27" s="52"/>
       <x:c r="C27" s="52"/>
@@ -5100,16 +5100,16 @@
         <x:v>证据一致性</x:v>
       </x:c>
       <x:c r="C30" s="27" t="str">
-        <x:v>每条关键结论都有直接支持它的证据</x:v>
+        <x:v>每条关键结论及待复核项中的事实前提都有直接支持证据</x:v>
       </x:c>
       <x:c r="D30" s="27" t="str">
-        <x:v>链接存在但页面不支持结论</x:v>
+        <x:v>链接存在但不支持结论，或待复核项暗含无依据事件</x:v>
       </x:c>
       <x:c r="E30" s="27" t="str">
         <x:v>需修改或失败</x:v>
       </x:c>
       <x:c r="F30" s="27" t="str">
-        <x:v>逐条对照结论与原文含义</x:v>
+        <x:v>逐条对照结论、未知项前提与原文含义</x:v>
       </x:c>
       <x:c r="G30" s="1"/>
       <x:c r="H30" s="1"/>
@@ -5174,16 +5174,16 @@
         <x:v>限制完整性</x:v>
       </x:c>
       <x:c r="C32" s="27" t="str">
-        <x:v>覆盖限制、失败模式、额度、可用性和量化评测</x:v>
+        <x:v>同时覆盖操作限制与模型质量失败模式；官方已披露时至少提取 2 项</x:v>
       </x:c>
       <x:c r="D32" s="27" t="str">
-        <x:v>只写优点，遗漏幻觉或错误推断</x:v>
+        <x:v>只写额度权限，遗漏幻觉、错误推断等质量问题</x:v>
       </x:c>
       <x:c r="E32" s="27" t="str">
         <x:v>需修改</x:v>
       </x:c>
       <x:c r="F32" s="27" t="str">
-        <x:v>主动寻找不利信息</x:v>
+        <x:v>操作限制不能替代模型质量限制</x:v>
       </x:c>
       <x:c r="G32" s="1"/>
       <x:c r="H32" s="1"/>
@@ -5211,16 +5211,16 @@
         <x:v>冲突与未知</x:v>
       </x:c>
       <x:c r="C33" s="27" t="str">
-        <x:v>冲突并列；无法确认写未知，不自行补全</x:v>
+        <x:v>冲突并列；未知项使用中性问题，不引入无依据事实前提</x:v>
       </x:c>
       <x:c r="D33" s="27" t="str">
-        <x:v>擅自裁决冲突或把未找到写成不存在</x:v>
+        <x:v>把未找到写成不存在，或假设某方案暂停后再询问影响</x:v>
       </x:c>
       <x:c r="E33" s="27" t="str">
         <x:v>需修改</x:v>
       </x:c>
       <x:c r="F33" s="27" t="str">
-        <x:v>检查否定性结论的证据</x:v>
+        <x:v>未知项若含事件前提，必须提供直接来源</x:v>
       </x:c>
       <x:c r="G33" s="1"/>
       <x:c r="H33" s="1"/>

</xml_diff>

<commit_message>
docs: record T001 v3 evidence failure
</commit_message>
<xml_diff>
--- a/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
+++ b/docs/product/DEERFLOW_EVALUATION_SCORECARD.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R366e3e5910494b15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="R7b4314fb6ef04914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="R11cd880bd93e498a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R548235e2263f4d44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测记录" sheetId="2" r:id="Rf3a5f9baa6924ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分标准" sheetId="3" r:id="R233149d3db154ac1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,7 +74,7 @@
       <x:name val="Microsoft YaHei"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -136,6 +136,16 @@
         <x:fgColor rgb="FFEEF4FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="4">
     <x:border/>
@@ -185,7 +195,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="66">
+  <x:cellXfs count="74">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -330,11 +340,35 @@
     <x:xf numFmtId="200" fontId="1" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="6">
+  <x:dxfs count="9">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -401,12 +435,45 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF0F5132"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD1E7DD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF842029"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF8D7DA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF664D03"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF3CD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvaluationTasks" displayName="EvaluationTasks" ref="A5:W11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvaluationTasks" displayName="EvaluationTasks" ref="A5:W12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="23">
     <x:tableColumn id="1" name="任务ID"/>
     <x:tableColumn id="2" name="用户场景"/>
@@ -766,33 +833,33 @@
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="15" t="n">
-        <x:f>COUNTA('评测记录'!$A$6:$A$11)</x:f>
-        <x:v>6</x:v>
+        <x:f>COUNTA('评测记录'!$A$6:$A$12)</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B5" s="15"/>
       <x:c r="C5" s="15" t="n">
-        <x:f>COUNTIFS('评测记录'!$F$6:$F$11,"已执行")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIFS('评测记录'!$F$6:$F$12,"已执行")</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D5" s="15"/>
       <x:c r="E5" s="16" t="n">
-        <x:f>IF(COUNT('评测记录'!$S$6:$S$11)=0,0,AVERAGE('评测记录'!$S$6:$S$11))</x:f>
-        <x:v>73</x:v>
+        <x:f>IF(COUNT('评测记录'!$S$6:$S$12)=0,0,AVERAGE('评测记录'!$S$6:$S$12))</x:f>
+        <x:v>60.666666666666664</x:v>
       </x:c>
       <x:c r="F5" s="16"/>
       <x:c r="G5" s="17" t="n">
-        <x:f>IF(COUNTIFS('评测记录'!$F$6:$F$11,"已执行")=0,0,COUNTIFS('评测记录'!$T$6:$T$11,"通过")/COUNTIFS('评测记录'!$F$6:$F$11,"已执行"))</x:f>
+        <x:f>IF(COUNTIFS('评测记录'!$F$6:$F$12,"已执行")=0,0,COUNTIFS('评测记录'!$T$6:$T$12,"通过")/COUNTIFS('评测记录'!$F$6:$F$12,"已执行"))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="17"/>
       <x:c r="I5" s="15" t="n">
-        <x:f>SUM('评测记录'!$P$6:$P$11)</x:f>
-        <x:v>76242</x:v>
+        <x:f>SUM('评测记录'!$P$6:$P$12)</x:f>
+        <x:v>125399</x:v>
       </x:c>
       <x:c r="J5" s="15"/>
       <x:c r="K5" s="18" t="n">
-        <x:f>SUM('评测记录'!$R$6:$R$11)</x:f>
-        <x:v>0.164736</x:v>
+        <x:f>SUM('评测记录'!$R$6:$R$12)</x:f>
+        <x:v>0.268792</x:v>
       </x:c>
       <x:c r="L5" s="18"/>
       <x:c r="M5" s="1"/>
@@ -1198,16 +1265,16 @@
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="27" t="str">
-        <x:v>质量门禁 v1.2 已修正</x:v>
+        <x:v>T001 v3 回归未通过</x:v>
       </x:c>
       <x:c r="B19" s="27" t="str">
-        <x:v>补充未知项前提检查，并强制区分操作限制与模型质量限制</x:v>
+        <x:v>未知项表述已改善，但关键来源读取与长度自检仍失败</x:v>
       </x:c>
       <x:c r="C19" s="27" t="str">
-        <x:v>T001 v3 尚未运行，v1.2 仅完成规则级验证</x:v>
+        <x:v>提示词规则不能稳定保证模型读取已访问页面中的证据</x:v>
       </x:c>
       <x:c r="D19" s="27" t="str">
-        <x:v>不执行 T002；获得新费用授权后再决定是否运行 T001 v3</x:v>
+        <x:v>停止追加付费样本；先设计确定性证据校验与人工发布闸门</x:v>
       </x:c>
       <x:c r="E19" s="1"/>
       <x:c r="F19" s="1"/>
@@ -2841,30 +2908,82 @@
         <x:v>Codex 辅助人工复核，2026-09-19。2 次搜索、3 次查看、3 个唯一官方页面；未见第三方来源、子智能体或文件生成。主回复输入约 32.4K、输出 900；线程顶部输入 32.7K、输出 909、总量 33.6K。延迟约 10 秒，正文 575 个总字符。较 v1 得分增加 12，主回复成本约下降 22%，正文长度约下降 55%。</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="1"/>
-      <x:c r="B12" s="1"/>
-      <x:c r="C12" s="1"/>
-      <x:c r="D12" s="1"/>
-      <x:c r="E12" s="1"/>
-      <x:c r="F12" s="1"/>
-      <x:c r="G12" s="1"/>
-      <x:c r="H12" s="1"/>
-      <x:c r="I12" s="1"/>
-      <x:c r="J12" s="1"/>
-      <x:c r="K12" s="1"/>
-      <x:c r="L12" s="1"/>
-      <x:c r="M12" s="1"/>
-      <x:c r="N12" s="1"/>
-      <x:c r="O12" s="1"/>
-      <x:c r="P12" s="1"/>
-      <x:c r="Q12" s="1"/>
-      <x:c r="R12" s="1"/>
-      <x:c r="S12" s="1"/>
-      <x:c r="T12" s="1"/>
-      <x:c r="U12" s="1"/>
-      <x:c r="V12" s="1"/>
-      <x:c r="W12" s="1"/>
+    <x:row r="12" ht="170" customHeight="1">
+      <x:c r="A12" s="28" t="str">
+        <x:v>T001-v3</x:v>
+      </x:c>
+      <x:c r="B12" s="27" t="str">
+        <x:v>关键限制提取与证据自检回归</x:v>
+      </x:c>
+      <x:c r="C12" s="27" t="str">
+        <x:v>按 RESEARCH_QUALITY_GATES.md 的 T001 v3 指令执行：最多 2 次搜索、3 个唯一官方页面，必须提取至少 2 项官方披露的模型质量失败模式，待复核项不得引入无依据前提，输出不超过 800 个总字符。</x:v>
+      </x:c>
+      <x:c r="D12" s="27" t="str">
+        <x:v>当前事实、历史信息、主要限制、待人工复核项</x:v>
+      </x:c>
+      <x:c r="E12" s="27" t="str">
+        <x:v>关键来源读取不完整、否定性结论与原文冲突、长度自检失真</x:v>
+      </x:c>
+      <x:c r="F12" s="70" t="str">
+        <x:v>已执行</x:v>
+      </x:c>
+      <x:c r="G12" s="70" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H12" s="70" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I12" s="70" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J12" s="70" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K12" s="70" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L12" s="70" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" s="70" t="str">
+        <x:v>需修改</x:v>
+      </x:c>
+      <x:c r="N12" s="70" t="n">
+        <x:v>48200</x:v>
+      </x:c>
+      <x:c r="O12" s="70" t="n">
+        <x:v>957</x:v>
+      </x:c>
+      <x:c r="P12" s="71" t="n">
+        <x:f>IF(COUNT(N12:O12)=0,"",SUM(N12:O12))</x:f>
+        <x:v>49157</x:v>
+      </x:c>
+      <x:c r="Q12" s="70" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="R12" s="72" t="n">
+        <x:f>IF(F12&lt;&gt;"已执行","",N12*'概览'!$B$9/1000000+O12*'概览'!$C$9/1000000)</x:f>
+        <x:v>0.104056</x:v>
+      </x:c>
+      <x:c r="S12" s="73" t="n">
+        <x:f>IF(COUNT(G12:K12)&lt;5,"",(G12*'评分标准'!$B$4+H12*'评分标准'!$B$5+I12*'评分标准'!$B$6+J12*'评分标准'!$B$7+K12*'评分标准'!$B$8)/5*100)</x:f>
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="T12" s="71" t="str">
+        <x:f>IF(F12&lt;&gt;"已执行","待执行",IF(L12&gt;0,"失败",IF(M12="失败","失败",IF(M12="需修改","需改进",IF(M12&lt;&gt;"通过","待人工复核",IF(S12&gt;=80,"通过","需改进"))))))</x:f>
+        <x:v>需改进</x:v>
+      </x:c>
+      <x:c r="U12" s="66" t="str">
+        <x:v>已正确区分当前与历史信息，也避免在待复核项中引入新事实前提；但在已查看官方发布页的 limitations 段后，仍错误声称页面未披露幻觉、错误推断、权威来源识别和置信度校准问题。关键否定性结论与来源原文冲突；可见正文 877 个总字符，却自报约 560 并声称符合 800 上限。</x:v>
+      </x:c>
+      <x:c r="V12" s="66" t="str">
+        <x:v>http://localhost:2026/workspace/chats/6604da82-dd28-47a2-9223-23f36fc31182
+https://help.openai.com/en/articles/10500283-deep-research-in-chatgpt
+https://openai.com/index/introducing-deep-research/</x:v>
+      </x:c>
+      <x:c r="W12" s="66" t="str">
+        <x:v>Codex 辅助人工复核，2026-09-19。2 次搜索、4 次页面查看；按去除 URL 片段计算 3 个唯一 URL，实质主要依赖 2 篇官方文章；未见第三方来源、子智能体或文件生成。主轮输入约 48.2K、输出 957、总量约 49.1K；线程顶部输入 48.5K、输出 965、总量 49.5K。UI 观测延迟约 5 秒。官方发布页 limitations 段明确列出幻觉、错误推断、权威来源识别和置信度校准问题，因此“未披露”结论错误。</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1"/>
@@ -4105,7 +4224,24 @@
     <x:cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="失败"/>
     <x:cfRule type="containsText" dxfId="5" priority="8" operator="containsText" text="需改进"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="12">
+  <x:conditionalFormatting sqref="S12:S12">
+    <x:cfRule type="colorScale" priority="9">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8D7DA"/>
+        <x:color rgb="FFFFF3CD"/>
+        <x:color rgb="FFD1E7DD"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="T12:T12">
+    <x:cfRule type="containsText" dxfId="6" priority="10" operator="containsText" text="通过"/>
+    <x:cfRule type="containsText" dxfId="7" priority="11" operator="containsText" text="失败"/>
+    <x:cfRule type="containsText" dxfId="8" priority="12" operator="containsText" text="需改进"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="18">
     <x:dataValidation type="list" sqref="F6:F10">
       <x:formula1>"未执行,已执行"</x:formula1>
     </x:dataValidation>
@@ -4146,10 +4282,30 @@
     <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="Q11">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="F12">
+      <x:formula1>"未执行,已执行"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="G12:K12">
+      <x:formula1>0</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="L12">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="M12">
+      <x:formula1>"待复核,通过,需修改,失败"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="N12:O12">
+      <x:formula1>0</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="Q12">
+      <x:formula1>0</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc0185037b7e4497"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa2aca9acdc849a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>